<commit_message>
feat: support up to 6+ images and multi-image color variants in excel parser and templates
</commit_message>
<xml_diff>
--- a/admin/public/gravoz_product_import_template.xlsx
+++ b/admin/public/gravoz_product_import_template.xlsx
@@ -397,29 +397,30 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:U4"/>
+  <dimension ref="A1:V3"/>
   <cols>
-    <col min="1" max="1" width="15.83203125" customWidth="1"/>
-    <col min="2" max="2" width="35.83203125" customWidth="1"/>
+    <col min="1" max="1" width="14.83203125" customWidth="1"/>
+    <col min="2" max="2" width="32.83203125" customWidth="1"/>
     <col min="3" max="3" width="16.83203125" customWidth="1"/>
-    <col min="4" max="4" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="20.83203125" customWidth="1"/>
     <col min="5" max="5" width="16.83203125" customWidth="1"/>
     <col min="6" max="6" width="10.83203125" customWidth="1"/>
     <col min="7" max="7" width="14.83203125" customWidth="1"/>
     <col min="8" max="8" width="10.83203125" customWidth="1"/>
     <col min="9" max="9" width="20.83203125" customWidth="1"/>
-    <col min="10" max="10" width="25.83203125" customWidth="1"/>
+    <col min="10" max="10" width="20.83203125" customWidth="1"/>
     <col min="11" max="11" width="45.83203125" customWidth="1"/>
     <col min="12" max="12" width="45.83203125" customWidth="1"/>
     <col min="13" max="13" width="45.83203125" customWidth="1"/>
     <col min="14" max="14" width="45.83203125" customWidth="1"/>
     <col min="15" max="15" width="45.83203125" customWidth="1"/>
-    <col min="16" max="16" width="50.83203125" customWidth="1"/>
-    <col min="17" max="17" width="35.83203125" customWidth="1"/>
-    <col min="18" max="18" width="50.83203125" customWidth="1"/>
-    <col min="19" max="19" width="14.83203125" customWidth="1"/>
+    <col min="16" max="16" width="45.83203125" customWidth="1"/>
+    <col min="17" max="17" width="60.83203125" customWidth="1"/>
+    <col min="18" max="18" width="35.83203125" customWidth="1"/>
+    <col min="19" max="19" width="50.83203125" customWidth="1"/>
     <col min="20" max="20" width="14.83203125" customWidth="1"/>
-    <col min="21" max="21" width="12.83203125" customWidth="1"/>
+    <col min="21" max="21" width="14.83203125" customWidth="1"/>
+    <col min="22" max="22" width="12.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -469,95 +470,101 @@
         <v>Image 5</v>
       </c>
       <c r="P1" t="str">
+        <v>Image 6</v>
+      </c>
+      <c r="Q1" t="str">
         <v>Color Variant Images</v>
       </c>
-      <c r="Q1" t="str">
+      <c r="R1" t="str">
         <v>Material</v>
       </c>
-      <c r="R1" t="str">
+      <c r="S1" t="str">
         <v>Description</v>
       </c>
-      <c r="S1" t="str">
+      <c r="T1" t="str">
         <v>Is Best Seller</v>
       </c>
-      <c r="T1" t="str">
+      <c r="U1" t="str">
         <v>Is Featured</v>
       </c>
-      <c r="U1" t="str">
+      <c r="V1" t="str">
         <v>Status</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>GRV-MEN-001</v>
+        <v>JS5061</v>
       </c>
       <c r="B2" t="str">
-        <v>Gravoz Apex Air Runner Shoes</v>
+        <v>Pure Leather Casual Shoe</v>
       </c>
       <c r="C2" t="str">
         <v>Men</v>
       </c>
       <c r="D2" t="str">
-        <v>Sports Shoes</v>
+        <v>Casual Shoe (Men)</v>
       </c>
       <c r="E2" t="str">
-        <v>Running</v>
+        <v>Casual Shoes</v>
       </c>
       <c r="F2">
-        <v>2999</v>
+        <v>1429</v>
       </c>
       <c r="G2">
-        <v>1499</v>
+        <v>1399</v>
       </c>
       <c r="H2">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="I2" t="str">
         <v>6, 7, 8, 9, 10, 11</v>
       </c>
       <c r="J2" t="str">
-        <v>Black, Olive, Grey</v>
+        <v>Brown, Black</v>
       </c>
       <c r="K2" t="str">
-        <v>https://images.unsplash.com/photo-1542291026-7eec264c27ff?w=800</v>
+        <v>https://images.unsplash.com/photo-1533867617858-e7b97e060509?w=800</v>
       </c>
       <c r="L2" t="str">
-        <v>https://images.unsplash.com/photo-1608231387042-66d1773070a5?w=800</v>
+        <v>https://images.unsplash.com/photo-1549298916-b41d501d3772?w=800</v>
       </c>
       <c r="M2" t="str">
+        <v>https://images.unsplash.com/photo-1560769629-975ec94e6a86?w=800</v>
+      </c>
+      <c r="N2" t="str">
         <v>https://images.unsplash.com/photo-1595950653106-6c9ebd614d3a?w=800</v>
-      </c>
-      <c r="N2" t="str">
-        <v>https://images.unsplash.com/photo-1525966222134-fcfa99b8ae77?w=800</v>
       </c>
       <c r="O2" t="str">
         <v>https://images.unsplash.com/photo-1584735935682-2f2b69dff9d2?w=800</v>
       </c>
       <c r="P2" t="str">
-        <v>Black:https://images.unsplash.com/photo-1542291026-7eec264c27ff?w=800; Olive:https://images.unsplash.com/photo-1608231387042-66d1773070a5?w=800</v>
+        <v>https://images.unsplash.com/photo-1608231387042-66d1773070a5?w=800</v>
       </c>
       <c r="Q2" t="str">
-        <v>Breathable Engineered Mesh &amp; Phylon Sole</v>
+        <v>Brown: https://images.unsplash.com/photo-1533867617858-e7b97e060509?w=800, https://images.unsplash.com/photo-1549298916-b41d501d3772?w=800 | Black: https://images.unsplash.com/photo-1525966222134-fcfa99b8ae77?w=800, https://images.unsplash.com/photo-1584735935682-2f2b69dff9d2?w=800</v>
       </c>
       <c r="R2" t="str">
-        <v>Ultra lightweight daily running shoes engineered with high rebound responsive cushioning.</v>
+        <v>Genuine Pure Leather &amp; Hand-Stitched Rubber Sole</v>
       </c>
       <c r="S2" t="str">
-        <v>TRUE</v>
+        <v>Premium handcrafted pure leather casual loafer shoes with soft cushioned footbed.</v>
       </c>
       <c r="T2" t="str">
         <v>TRUE</v>
       </c>
       <c r="U2" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="V2" t="str">
         <v>active</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>GRV-WMN-002</v>
+        <v>GRV-WMN-02</v>
       </c>
       <c r="B3" t="str">
-        <v>Gravoz FeatherLite Walking Sneaker</v>
+        <v>Gravoz CloudComfort Slip-on Loafer</v>
       </c>
       <c r="C3" t="str">
         <v>Women</v>
@@ -566,7 +573,7 @@
         <v>Casual Footwear</v>
       </c>
       <c r="E3" t="str">
-        <v>Walking</v>
+        <v>Loafers</v>
       </c>
       <c r="F3">
         <v>2499</v>
@@ -581,7 +588,7 @@
         <v>4, 5, 6, 7, 8</v>
       </c>
       <c r="J3" t="str">
-        <v>Blush Pink, Pure White, Lavender</v>
+        <v>Tan, Beige, Black</v>
       </c>
       <c r="K3" t="str">
         <v>https://images.unsplash.com/photo-1560769629-975ec94e6a86?w=800</v>
@@ -599,92 +606,30 @@
         <v>https://images.unsplash.com/photo-1539185441755-769473a23570?w=800</v>
       </c>
       <c r="P3" t="str">
-        <v>Blush Pink:https://images.unsplash.com/photo-1560769629-975ec94e6a86?w=800; Pure White:https://images.unsplash.com/photo-1595341888016-a392ef81b7de?w=800</v>
+        <v/>
       </c>
       <c r="Q3" t="str">
-        <v>Soft Stretch Knit with Memory Foam Insole</v>
+        <v>Tan: https://images.unsplash.com/photo-1560769629-975ec94e6a86?w=800 | Beige: https://images.unsplash.com/photo-1595341888016-a392ef81b7de?w=800</v>
       </c>
       <c r="R3" t="str">
+        <v>Soft Stretch Suede Leather</v>
+      </c>
+      <c r="S3" t="str">
         <v>Ergonomic slip-on walking shoes designed for maximum all-day comfort and arch support.</v>
-      </c>
-      <c r="S3" t="str">
-        <v>TRUE</v>
       </c>
       <c r="T3" t="str">
         <v>TRUE</v>
       </c>
       <c r="U3" t="str">
-        <v>active</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>GRV-KID-003</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Gravoz PlayGround Flex Kids Runner</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Babies</v>
-      </c>
-      <c r="D4" t="str">
-        <v>Kids Footwear</v>
-      </c>
-      <c r="E4" t="str">
-        <v>Sports</v>
-      </c>
-      <c r="F4">
-        <v>1899</v>
-      </c>
-      <c r="G4">
-        <v>999</v>
-      </c>
-      <c r="H4">
-        <v>60</v>
-      </c>
-      <c r="I4" t="str">
-        <v>1, 2, 3, 4, 5</v>
-      </c>
-      <c r="J4" t="str">
-        <v>Royal Blue, Sunset Orange</v>
-      </c>
-      <c r="K4" t="str">
-        <v>https://images.unsplash.com/photo-1514989940723-e8e51635b782?w=800</v>
-      </c>
-      <c r="L4" t="str">
-        <v>https://images.unsplash.com/photo-1509255673980-ed8101dd25f9?w=800</v>
-      </c>
-      <c r="M4" t="str">
-        <v>https://images.unsplash.com/photo-1511556532299-8f662fc26c06?w=800</v>
-      </c>
-      <c r="N4" t="str">
-        <v/>
-      </c>
-      <c r="O4" t="str">
-        <v/>
-      </c>
-      <c r="P4" t="str">
-        <v>Royal Blue:https://images.unsplash.com/photo-1514989940723-e8e51635b782?w=800</v>
-      </c>
-      <c r="Q4" t="str">
-        <v>Durable Canvas with Non-Slip Grip Sole</v>
-      </c>
-      <c r="R4" t="str">
-        <v>Lightweight easy-wear hook and loop strap sneakers for active boys and girls.</v>
-      </c>
-      <c r="S4" t="str">
-        <v>FALSE</v>
-      </c>
-      <c r="T4" t="str">
         <v>TRUE</v>
       </c>
-      <c r="U4" t="str">
+      <c r="V3" t="str">
         <v>active</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:U4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:V3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(importer): add 10-image dual color variant template and per-color column auto-mapper
</commit_message>
<xml_diff>
--- a/admin/public/gravoz_product_import_template.xlsx
+++ b/admin/public/gravoz_product_import_template.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Products Template" sheetId="1" r:id="rId1"/>
+    <sheet name="Products Template (10 Images)" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:V3"/>
+  <dimension ref="A1:AD3"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="32.83203125" customWidth="1"/>
@@ -408,19 +408,22 @@
     <col min="7" max="7" width="14.83203125" customWidth="1"/>
     <col min="8" max="8" width="10.83203125" customWidth="1"/>
     <col min="9" max="9" width="20.83203125" customWidth="1"/>
-    <col min="10" max="10" width="20.83203125" customWidth="1"/>
+    <col min="10" max="10" width="16.83203125" customWidth="1"/>
     <col min="11" max="11" width="45.83203125" customWidth="1"/>
     <col min="12" max="12" width="45.83203125" customWidth="1"/>
     <col min="13" max="13" width="45.83203125" customWidth="1"/>
     <col min="14" max="14" width="45.83203125" customWidth="1"/>
     <col min="15" max="15" width="45.83203125" customWidth="1"/>
     <col min="16" max="16" width="45.83203125" customWidth="1"/>
-    <col min="17" max="17" width="60.83203125" customWidth="1"/>
-    <col min="18" max="18" width="35.83203125" customWidth="1"/>
-    <col min="19" max="19" width="50.83203125" customWidth="1"/>
-    <col min="20" max="20" width="14.83203125" customWidth="1"/>
-    <col min="21" max="21" width="14.83203125" customWidth="1"/>
-    <col min="22" max="22" width="12.83203125" customWidth="1"/>
+    <col min="17" max="17" width="45.83203125" customWidth="1"/>
+    <col min="18" max="18" width="45.83203125" customWidth="1"/>
+    <col min="19" max="19" width="45.83203125" customWidth="1"/>
+    <col min="20" max="20" width="45.83203125" customWidth="1"/>
+    <col min="21" max="21" width="40.83203125" customWidth="1"/>
+    <col min="22" max="22" width="50.83203125" customWidth="1"/>
+    <col min="23" max="23" width="14.83203125" customWidth="1"/>
+    <col min="24" max="24" width="14.83203125" customWidth="1"/>
+    <col min="25" max="25" width="12.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -455,40 +458,64 @@
         <v>Colors</v>
       </c>
       <c r="K1" t="str">
-        <v>Image 1</v>
+        <v>Brown Image 1</v>
       </c>
       <c r="L1" t="str">
-        <v>Image 2</v>
+        <v>Brown Image 2</v>
       </c>
       <c r="M1" t="str">
-        <v>Image 3</v>
+        <v>Brown Image 3</v>
       </c>
       <c r="N1" t="str">
-        <v>Image 4</v>
+        <v>Brown Image 4</v>
       </c>
       <c r="O1" t="str">
-        <v>Image 5</v>
+        <v>Brown Image 5</v>
       </c>
       <c r="P1" t="str">
-        <v>Image 6</v>
+        <v>Black Image 1</v>
       </c>
       <c r="Q1" t="str">
-        <v>Color Variant Images</v>
+        <v>Black Image 2</v>
       </c>
       <c r="R1" t="str">
+        <v>Black Image 3</v>
+      </c>
+      <c r="S1" t="str">
+        <v>Black Image 4</v>
+      </c>
+      <c r="T1" t="str">
+        <v>Black Image 5</v>
+      </c>
+      <c r="U1" t="str">
         <v>Material</v>
       </c>
-      <c r="S1" t="str">
+      <c r="V1" t="str">
         <v>Description</v>
       </c>
-      <c r="T1" t="str">
+      <c r="W1" t="str">
         <v>Is Best Seller</v>
       </c>
-      <c r="U1" t="str">
+      <c r="X1" t="str">
         <v>Is Featured</v>
       </c>
-      <c r="V1" t="str">
+      <c r="Y1" t="str">
         <v>Status</v>
+      </c>
+      <c r="Z1" t="str">
+        <v>Tan Image 1</v>
+      </c>
+      <c r="AA1" t="str">
+        <v>Tan Image 2</v>
+      </c>
+      <c r="AB1" t="str">
+        <v>Tan Image 3</v>
+      </c>
+      <c r="AC1" t="str">
+        <v>Tan Image 4</v>
+      </c>
+      <c r="AD1" t="str">
+        <v>Tan Image 5</v>
       </c>
     </row>
     <row r="2">
@@ -538,98 +565,116 @@
         <v>https://images.unsplash.com/photo-1584735935682-2f2b69dff9d2?w=800</v>
       </c>
       <c r="P2" t="str">
+        <v>https://images.unsplash.com/photo-1525966222134-fcfa99b8ae77?w=800</v>
+      </c>
+      <c r="Q2" t="str">
+        <v>https://images.unsplash.com/photo-1514989940723-e8e51635b782?w=800</v>
+      </c>
+      <c r="R2" t="str">
+        <v>https://images.unsplash.com/photo-1512374382149-233c42b661ac?w=800</v>
+      </c>
+      <c r="S2" t="str">
         <v>https://images.unsplash.com/photo-1608231387042-66d1773070a5?w=800</v>
       </c>
-      <c r="Q2" t="str">
-        <v>Brown: https://images.unsplash.com/photo-1533867617858-e7b97e060509?w=800, https://images.unsplash.com/photo-1549298916-b41d501d3772?w=800 | Black: https://images.unsplash.com/photo-1525966222134-fcfa99b8ae77?w=800, https://images.unsplash.com/photo-1584735935682-2f2b69dff9d2?w=800</v>
-      </c>
-      <c r="R2" t="str">
+      <c r="T2" t="str">
+        <v>https://images.unsplash.com/photo-1539185441755-769473a23570?w=800</v>
+      </c>
+      <c r="U2" t="str">
         <v>Genuine Pure Leather &amp; Hand-Stitched Rubber Sole</v>
       </c>
-      <c r="S2" t="str">
+      <c r="V2" t="str">
         <v>Premium handcrafted pure leather casual loafer shoes with soft cushioned footbed.</v>
       </c>
-      <c r="T2" t="str">
+      <c r="W2" t="str">
         <v>TRUE</v>
       </c>
-      <c r="U2" t="str">
+      <c r="X2" t="str">
         <v>TRUE</v>
       </c>
-      <c r="V2" t="str">
+      <c r="Y2" t="str">
         <v>active</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>GRV-WMN-02</v>
+        <v>JS5062</v>
       </c>
       <c r="B3" t="str">
-        <v>Gravoz CloudComfort Slip-on Loafer</v>
+        <v>Italian Classic Oxford Formal</v>
       </c>
       <c r="C3" t="str">
-        <v>Women</v>
+        <v>Men</v>
       </c>
       <c r="D3" t="str">
-        <v>Casual Footwear</v>
+        <v>Formal Shoes</v>
       </c>
       <c r="E3" t="str">
-        <v>Loafers</v>
+        <v>Oxford</v>
       </c>
       <c r="F3">
         <v>2499</v>
       </c>
       <c r="G3">
-        <v>1299</v>
+        <v>1999</v>
       </c>
       <c r="H3">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="I3" t="str">
-        <v>4, 5, 6, 7, 8</v>
+        <v>7, 8, 9, 10, 11</v>
       </c>
       <c r="J3" t="str">
-        <v>Tan, Beige, Black</v>
-      </c>
-      <c r="K3" t="str">
+        <v>Tan, Black</v>
+      </c>
+      <c r="P3" t="str">
+        <v>https://images.unsplash.com/photo-1543163521-1bf539c55dd2?w=800</v>
+      </c>
+      <c r="Q3" t="str">
+        <v>https://images.unsplash.com/photo-1525966222134-fcfa99b8ae77?w=800</v>
+      </c>
+      <c r="R3" t="str">
+        <v>https://images.unsplash.com/photo-1512374382149-233c42b661ac?w=800</v>
+      </c>
+      <c r="S3" t="str">
+        <v>https://images.unsplash.com/photo-1608231387042-66d1773070a5?w=800</v>
+      </c>
+      <c r="T3" t="str">
+        <v>https://images.unsplash.com/photo-1539185441755-769473a23570?w=800</v>
+      </c>
+      <c r="U3" t="str">
+        <v>Full Grain Italian Leather</v>
+      </c>
+      <c r="V3" t="str">
+        <v>Handmade genuine leather formal dress shoes for business and black-tie occasions.</v>
+      </c>
+      <c r="W3" t="str">
+        <v>FALSE</v>
+      </c>
+      <c r="X3" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="Y3" t="str">
+        <v>active</v>
+      </c>
+      <c r="Z3" t="str">
+        <v>https://images.unsplash.com/photo-1614252235316-8c857d38b5f4?w=800</v>
+      </c>
+      <c r="AA3" t="str">
+        <v>https://images.unsplash.com/photo-1533867617858-e7b97e060509?w=800</v>
+      </c>
+      <c r="AB3" t="str">
         <v>https://images.unsplash.com/photo-1560769629-975ec94e6a86?w=800</v>
       </c>
-      <c r="L3" t="str">
-        <v>https://images.unsplash.com/photo-1595341888016-a392ef81b7de?w=800</v>
-      </c>
-      <c r="M3" t="str">
-        <v>https://images.unsplash.com/photo-1512374382149-233c42b661ac?w=800</v>
-      </c>
-      <c r="N3" t="str">
-        <v>https://images.unsplash.com/photo-1515955656352-a1fa3ffcd111?w=800</v>
-      </c>
-      <c r="O3" t="str">
-        <v>https://images.unsplash.com/photo-1539185441755-769473a23570?w=800</v>
-      </c>
-      <c r="P3" t="str">
-        <v/>
-      </c>
-      <c r="Q3" t="str">
-        <v>Tan: https://images.unsplash.com/photo-1560769629-975ec94e6a86?w=800 | Beige: https://images.unsplash.com/photo-1595341888016-a392ef81b7de?w=800</v>
-      </c>
-      <c r="R3" t="str">
-        <v>Soft Stretch Suede Leather</v>
-      </c>
-      <c r="S3" t="str">
-        <v>Ergonomic slip-on walking shoes designed for maximum all-day comfort and arch support.</v>
-      </c>
-      <c r="T3" t="str">
-        <v>TRUE</v>
-      </c>
-      <c r="U3" t="str">
-        <v>TRUE</v>
-      </c>
-      <c r="V3" t="str">
-        <v>active</v>
+      <c r="AC3" t="str">
+        <v>https://images.unsplash.com/photo-1549298916-b41d501d3772?w=800</v>
+      </c>
+      <c r="AD3" t="str">
+        <v>https://images.unsplash.com/photo-1584735935682-2f2b69dff9d2?w=800</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:V3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AD3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update Excel product import template with clean per-color image columns (Method 1)
</commit_message>
<xml_diff>
--- a/admin/public/gravoz_product_import_template.xlsx
+++ b/admin/public/gravoz_product_import_template.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Products Template (10 Images)" sheetId="1" r:id="rId1"/>
+    <sheet name="Products" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,41 +397,31 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AD3"/>
+  <dimension ref="A1:O3"/>
   <cols>
-    <col min="1" max="1" width="14.83203125" customWidth="1"/>
-    <col min="2" max="2" width="32.83203125" customWidth="1"/>
-    <col min="3" max="3" width="16.83203125" customWidth="1"/>
-    <col min="4" max="4" width="20.83203125" customWidth="1"/>
+    <col min="1" max="1" width="28.83203125" customWidth="1"/>
+    <col min="2" max="2" width="15.83203125" customWidth="1"/>
+    <col min="3" max="3" width="15.83203125" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" customWidth="1"/>
     <col min="5" max="5" width="16.83203125" customWidth="1"/>
     <col min="6" max="6" width="10.83203125" customWidth="1"/>
     <col min="7" max="7" width="14.83203125" customWidth="1"/>
-    <col min="8" max="8" width="10.83203125" customWidth="1"/>
-    <col min="9" max="9" width="20.83203125" customWidth="1"/>
-    <col min="10" max="10" width="16.83203125" customWidth="1"/>
-    <col min="11" max="11" width="45.83203125" customWidth="1"/>
-    <col min="12" max="12" width="45.83203125" customWidth="1"/>
-    <col min="13" max="13" width="45.83203125" customWidth="1"/>
-    <col min="14" max="14" width="45.83203125" customWidth="1"/>
+    <col min="8" max="8" width="8.83203125" customWidth="1"/>
+    <col min="9" max="9" width="18.83203125" customWidth="1"/>
+    <col min="10" max="10" width="20.83203125" customWidth="1"/>
+    <col min="11" max="11" width="55.83203125" customWidth="1"/>
+    <col min="12" max="12" width="55.83203125" customWidth="1"/>
+    <col min="13" max="13" width="55.83203125" customWidth="1"/>
+    <col min="14" max="14" width="20.83203125" customWidth="1"/>
     <col min="15" max="15" width="45.83203125" customWidth="1"/>
-    <col min="16" max="16" width="45.83203125" customWidth="1"/>
-    <col min="17" max="17" width="45.83203125" customWidth="1"/>
-    <col min="18" max="18" width="45.83203125" customWidth="1"/>
-    <col min="19" max="19" width="45.83203125" customWidth="1"/>
-    <col min="20" max="20" width="45.83203125" customWidth="1"/>
-    <col min="21" max="21" width="40.83203125" customWidth="1"/>
-    <col min="22" max="22" width="50.83203125" customWidth="1"/>
-    <col min="23" max="23" width="14.83203125" customWidth="1"/>
-    <col min="24" max="24" width="14.83203125" customWidth="1"/>
-    <col min="25" max="25" width="12.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
+        <v>Name</v>
+      </c>
+      <c r="B1" t="str">
         <v>SKU</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Name</v>
       </c>
       <c r="C1" t="str">
         <v>Target Audience</v>
@@ -458,223 +448,118 @@
         <v>Colors</v>
       </c>
       <c r="K1" t="str">
-        <v>Brown Image 1</v>
+        <v>Brown Images</v>
       </c>
       <c r="L1" t="str">
-        <v>Brown Image 2</v>
+        <v>Black Images</v>
       </c>
       <c r="M1" t="str">
-        <v>Brown Image 3</v>
+        <v>Tan Images</v>
       </c>
       <c r="N1" t="str">
-        <v>Brown Image 4</v>
+        <v>Material</v>
       </c>
       <c r="O1" t="str">
-        <v>Brown Image 5</v>
-      </c>
-      <c r="P1" t="str">
-        <v>Black Image 1</v>
-      </c>
-      <c r="Q1" t="str">
-        <v>Black Image 2</v>
-      </c>
-      <c r="R1" t="str">
-        <v>Black Image 3</v>
-      </c>
-      <c r="S1" t="str">
-        <v>Black Image 4</v>
-      </c>
-      <c r="T1" t="str">
-        <v>Black Image 5</v>
-      </c>
-      <c r="U1" t="str">
-        <v>Material</v>
-      </c>
-      <c r="V1" t="str">
         <v>Description</v>
-      </c>
-      <c r="W1" t="str">
-        <v>Is Best Seller</v>
-      </c>
-      <c r="X1" t="str">
-        <v>Is Featured</v>
-      </c>
-      <c r="Y1" t="str">
-        <v>Status</v>
-      </c>
-      <c r="Z1" t="str">
-        <v>Tan Image 1</v>
-      </c>
-      <c r="AA1" t="str">
-        <v>Tan Image 2</v>
-      </c>
-      <c r="AB1" t="str">
-        <v>Tan Image 3</v>
-      </c>
-      <c r="AC1" t="str">
-        <v>Tan Image 4</v>
-      </c>
-      <c r="AD1" t="str">
-        <v>Tan Image 5</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>JS5061</v>
+        <v>GRAVOZ EI Leather Sandals</v>
       </c>
       <c r="B2" t="str">
-        <v>Pure Leather Casual Shoe</v>
+        <v>GRV-EI-001</v>
       </c>
       <c r="C2" t="str">
         <v>Men</v>
       </c>
       <c r="D2" t="str">
-        <v>Casual Shoe (Men)</v>
+        <v>Sandals</v>
       </c>
       <c r="E2" t="str">
-        <v>Casual Shoes</v>
+        <v>Casual Sandals</v>
       </c>
       <c r="F2">
-        <v>1429</v>
+        <v>1399</v>
       </c>
       <c r="G2">
-        <v>1399</v>
+        <v>1199</v>
       </c>
       <c r="H2">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="I2" t="str">
         <v>6, 7, 8, 9, 10, 11</v>
       </c>
       <c r="J2" t="str">
-        <v>Brown, Black</v>
+        <v>Brown, Black, Tan</v>
       </c>
       <c r="K2" t="str">
-        <v>https://images.unsplash.com/photo-1533867617858-e7b97e060509?w=800</v>
+        <v>https://images.unsplash.com/photo-1533867617858-e7b97e060509?w=800, https://images.unsplash.com/photo-1549298916-b41d501d3772?w=800</v>
       </c>
       <c r="L2" t="str">
-        <v>https://images.unsplash.com/photo-1549298916-b41d501d3772?w=800</v>
+        <v>https://images.unsplash.com/photo-1525966222134-fcfa99b8ae77?w=800, https://images.unsplash.com/photo-1514989940723-e8e51635b782?w=800</v>
       </c>
       <c r="M2" t="str">
-        <v>https://images.unsplash.com/photo-1560769629-975ec94e6a86?w=800</v>
+        <v>https://images.unsplash.com/photo-1543163521-1bf539c55dd2?w=800, https://images.unsplash.com/photo-1560769629-975ec94e6a86?w=800</v>
       </c>
       <c r="N2" t="str">
-        <v>https://images.unsplash.com/photo-1595950653106-6c9ebd614d3a?w=800</v>
+        <v>Genuine Leather</v>
       </c>
       <c r="O2" t="str">
-        <v>https://images.unsplash.com/photo-1584735935682-2f2b69dff9d2?w=800</v>
-      </c>
-      <c r="P2" t="str">
-        <v>https://images.unsplash.com/photo-1525966222134-fcfa99b8ae77?w=800</v>
-      </c>
-      <c r="Q2" t="str">
-        <v>https://images.unsplash.com/photo-1514989940723-e8e51635b782?w=800</v>
-      </c>
-      <c r="R2" t="str">
-        <v>https://images.unsplash.com/photo-1512374382149-233c42b661ac?w=800</v>
-      </c>
-      <c r="S2" t="str">
-        <v>https://images.unsplash.com/photo-1608231387042-66d1773070a5?w=800</v>
-      </c>
-      <c r="T2" t="str">
-        <v>https://images.unsplash.com/photo-1539185441755-769473a23570?w=800</v>
-      </c>
-      <c r="U2" t="str">
-        <v>Genuine Pure Leather &amp; Hand-Stitched Rubber Sole</v>
-      </c>
-      <c r="V2" t="str">
-        <v>Premium handcrafted pure leather casual loafer shoes with soft cushioned footbed.</v>
-      </c>
-      <c r="W2" t="str">
-        <v>TRUE</v>
-      </c>
-      <c r="X2" t="str">
-        <v>TRUE</v>
-      </c>
-      <c r="Y2" t="str">
-        <v>active</v>
+        <v>Handcrafted premium leather sandals designed for all-day comfort.</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>JS5062</v>
+        <v>GRAVOZ Classic Derby Loafers</v>
       </c>
       <c r="B3" t="str">
-        <v>Italian Classic Oxford Formal</v>
+        <v>GRV-DERBY-002</v>
       </c>
       <c r="C3" t="str">
         <v>Men</v>
       </c>
       <c r="D3" t="str">
-        <v>Formal Shoes</v>
+        <v>Formal</v>
       </c>
       <c r="E3" t="str">
-        <v>Oxford</v>
+        <v>Loafers</v>
       </c>
       <c r="F3">
         <v>2499</v>
       </c>
       <c r="G3">
-        <v>1999</v>
+        <v>2199</v>
       </c>
       <c r="H3">
         <v>40</v>
       </c>
       <c r="I3" t="str">
-        <v>7, 8, 9, 10, 11</v>
+        <v>7, 8, 9, 10</v>
       </c>
       <c r="J3" t="str">
-        <v>Tan, Black</v>
-      </c>
-      <c r="P3" t="str">
-        <v>https://images.unsplash.com/photo-1543163521-1bf539c55dd2?w=800</v>
-      </c>
-      <c r="Q3" t="str">
-        <v>https://images.unsplash.com/photo-1525966222134-fcfa99b8ae77?w=800</v>
-      </c>
-      <c r="R3" t="str">
-        <v>https://images.unsplash.com/photo-1512374382149-233c42b661ac?w=800</v>
-      </c>
-      <c r="S3" t="str">
-        <v>https://images.unsplash.com/photo-1608231387042-66d1773070a5?w=800</v>
-      </c>
-      <c r="T3" t="str">
-        <v>https://images.unsplash.com/photo-1539185441755-769473a23570?w=800</v>
-      </c>
-      <c r="U3" t="str">
-        <v>Full Grain Italian Leather</v>
-      </c>
-      <c r="V3" t="str">
-        <v>Handmade genuine leather formal dress shoes for business and black-tie occasions.</v>
-      </c>
-      <c r="W3" t="str">
-        <v>FALSE</v>
-      </c>
-      <c r="X3" t="str">
-        <v>TRUE</v>
-      </c>
-      <c r="Y3" t="str">
-        <v>active</v>
-      </c>
-      <c r="Z3" t="str">
-        <v>https://images.unsplash.com/photo-1614252235316-8c857d38b5f4?w=800</v>
-      </c>
-      <c r="AA3" t="str">
-        <v>https://images.unsplash.com/photo-1533867617858-e7b97e060509?w=800</v>
-      </c>
-      <c r="AB3" t="str">
-        <v>https://images.unsplash.com/photo-1560769629-975ec94e6a86?w=800</v>
-      </c>
-      <c r="AC3" t="str">
-        <v>https://images.unsplash.com/photo-1549298916-b41d501d3772?w=800</v>
-      </c>
-      <c r="AD3" t="str">
-        <v>https://images.unsplash.com/photo-1584735935682-2f2b69dff9d2?w=800</v>
+        <v>Brown, Black</v>
+      </c>
+      <c r="K3" t="str">
+        <v>https://images.unsplash.com/photo-1533867617858-e7b97e060509?w=800, https://images.unsplash.com/photo-1549298916-b41d501d3772?w=800</v>
+      </c>
+      <c r="L3" t="str">
+        <v>https://images.unsplash.com/photo-1525966222134-fcfa99b8ae77?w=800, https://images.unsplash.com/photo-1514989940723-e8e51635b782?w=800</v>
+      </c>
+      <c r="M3" t="str">
+        <v/>
+      </c>
+      <c r="N3" t="str">
+        <v>Full Grain Leather</v>
+      </c>
+      <c r="O3" t="str">
+        <v>Elegant formal Derby shoes crafted from hand-selected full grain leather.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AD3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>